<commit_message>
Split card template into separate face and back sheets
</commit_message>
<xml_diff>
--- a/templates/card_template.xlsx
+++ b/templates/card_template.xlsx
@@ -7,8 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="стр.1" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="стр.2" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Лицевая сторона" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Оборотная сторона" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -82,7 +82,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -110,6 +110,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -481,17 +484,17 @@
   <dimension ref="A1:K37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -816,24 +819,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K29"/>
+  <dimension ref="A1:J24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
-    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="H1" s="4" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Оборотная сторона личной карточки</t>
         </is>
@@ -847,7 +849,7 @@
       </c>
       <c r="B3" s="8" t="inlineStr">
         <is>
-          <t>Модель, марка, артикул, класс защиты СИЗ</t>
+          <t>Модель, марка, артикул, класс защиты СИЗ, дерматологических СИЗ</t>
         </is>
       </c>
       <c r="C3" s="8" t="inlineStr">
@@ -858,15 +860,14 @@
       <c r="D3" s="8" t="n"/>
       <c r="E3" s="8" t="n"/>
       <c r="F3" s="8" t="n"/>
-      <c r="G3" s="8" t="n"/>
-      <c r="H3" s="8" t="inlineStr">
+      <c r="G3" s="8" t="inlineStr">
         <is>
           <t>Возвращено</t>
         </is>
       </c>
+      <c r="H3" s="8" t="n"/>
       <c r="I3" s="8" t="n"/>
       <c r="J3" s="8" t="n"/>
-      <c r="K3" s="8" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="8" t="n"/>
@@ -883,8 +884,8 @@
       </c>
       <c r="E4" s="8" t="inlineStr">
         <is>
-          <t>Лично/
-дозатор</t>
+          <t>Лично /
+карточка</t>
         </is>
       </c>
       <c r="F4" s="8" t="inlineStr">
@@ -894,27 +895,22 @@
       </c>
       <c r="G4" s="8" t="inlineStr">
         <is>
-          <t>подпись выдавшего</t>
+          <t>дата</t>
         </is>
       </c>
       <c r="H4" s="8" t="inlineStr">
         <is>
-          <t>дата</t>
+          <t>количество</t>
         </is>
       </c>
       <c r="I4" s="8" t="inlineStr">
         <is>
-          <t>количество</t>
+          <t>подпись сдавшего СИЗ</t>
         </is>
       </c>
       <c r="J4" s="8" t="inlineStr">
         <is>
-          <t>подпись сдавшего СИЗ</t>
-        </is>
-      </c>
-      <c r="K4" s="8" t="inlineStr">
-        <is>
-          <t>Акт списания (дата, номер)</t>
+          <t>Акт списания, дата и номер</t>
         </is>
       </c>
     </row>
@@ -949,279 +945,196 @@
       <c r="J5" s="8" t="n">
         <v>10</v>
       </c>
-      <c r="K5" s="8" t="n">
-        <v>11</v>
-      </c>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="n"/>
-      <c r="B6" s="11" t="n"/>
-      <c r="C6" s="11" t="n"/>
-      <c r="D6" s="11" t="n"/>
-      <c r="E6" s="11" t="n"/>
-      <c r="F6" s="11" t="n"/>
-      <c r="G6" s="11" t="n"/>
-      <c r="H6" s="11" t="n"/>
-      <c r="I6" s="11" t="n"/>
-      <c r="J6" s="11" t="n"/>
-      <c r="K6" s="11" t="n"/>
+      <c r="A6" s="12" t="n"/>
+      <c r="B6" s="12" t="n"/>
+      <c r="C6" s="12" t="n"/>
+      <c r="D6" s="12" t="n"/>
+      <c r="E6" s="12" t="n"/>
+      <c r="F6" s="12" t="n"/>
+      <c r="G6" s="12" t="n"/>
+      <c r="H6" s="12" t="n"/>
+      <c r="I6" s="12" t="n"/>
+      <c r="J6" s="12" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="n"/>
-      <c r="B7" s="11" t="n"/>
-      <c r="C7" s="11" t="n"/>
-      <c r="D7" s="11" t="n"/>
-      <c r="E7" s="11" t="n"/>
-      <c r="F7" s="11" t="n"/>
-      <c r="G7" s="11" t="n"/>
-      <c r="H7" s="11" t="n"/>
-      <c r="I7" s="11" t="n"/>
-      <c r="J7" s="11" t="n"/>
-      <c r="K7" s="11" t="n"/>
+      <c r="A7" s="12" t="n"/>
+      <c r="B7" s="12" t="n"/>
+      <c r="C7" s="12" t="n"/>
+      <c r="D7" s="12" t="n"/>
+      <c r="E7" s="12" t="n"/>
+      <c r="F7" s="12" t="n"/>
+      <c r="G7" s="12" t="n"/>
+      <c r="H7" s="12" t="n"/>
+      <c r="I7" s="12" t="n"/>
+      <c r="J7" s="12" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="11" t="n"/>
-      <c r="B8" s="11" t="n"/>
-      <c r="C8" s="11" t="n"/>
-      <c r="D8" s="11" t="n"/>
-      <c r="E8" s="11" t="n"/>
-      <c r="F8" s="11" t="n"/>
-      <c r="G8" s="11" t="n"/>
-      <c r="H8" s="11" t="n"/>
-      <c r="I8" s="11" t="n"/>
-      <c r="J8" s="11" t="n"/>
-      <c r="K8" s="11" t="n"/>
+      <c r="A8" s="12" t="n"/>
+      <c r="B8" s="12" t="n"/>
+      <c r="C8" s="12" t="n"/>
+      <c r="D8" s="12" t="n"/>
+      <c r="E8" s="12" t="n"/>
+      <c r="F8" s="12" t="n"/>
+      <c r="G8" s="12" t="n"/>
+      <c r="H8" s="12" t="n"/>
+      <c r="I8" s="12" t="n"/>
+      <c r="J8" s="12" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="11" t="n"/>
-      <c r="B9" s="11" t="n"/>
-      <c r="C9" s="11" t="n"/>
-      <c r="D9" s="11" t="n"/>
-      <c r="E9" s="11" t="n"/>
-      <c r="F9" s="11" t="n"/>
-      <c r="G9" s="11" t="n"/>
-      <c r="H9" s="11" t="n"/>
-      <c r="I9" s="11" t="n"/>
-      <c r="J9" s="11" t="n"/>
-      <c r="K9" s="11" t="n"/>
+      <c r="A9" s="12" t="n"/>
+      <c r="B9" s="12" t="n"/>
+      <c r="C9" s="12" t="n"/>
+      <c r="D9" s="12" t="n"/>
+      <c r="E9" s="12" t="n"/>
+      <c r="F9" s="12" t="n"/>
+      <c r="G9" s="12" t="n"/>
+      <c r="H9" s="12" t="n"/>
+      <c r="I9" s="12" t="n"/>
+      <c r="J9" s="12" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="11" t="n"/>
-      <c r="B10" s="11" t="n"/>
-      <c r="C10" s="11" t="n"/>
-      <c r="D10" s="11" t="n"/>
-      <c r="E10" s="11" t="n"/>
-      <c r="F10" s="11" t="n"/>
-      <c r="G10" s="11" t="n"/>
-      <c r="H10" s="11" t="n"/>
-      <c r="I10" s="11" t="n"/>
-      <c r="J10" s="11" t="n"/>
-      <c r="K10" s="11" t="n"/>
+      <c r="A10" s="12" t="n"/>
+      <c r="B10" s="12" t="n"/>
+      <c r="C10" s="12" t="n"/>
+      <c r="D10" s="12" t="n"/>
+      <c r="E10" s="12" t="n"/>
+      <c r="F10" s="12" t="n"/>
+      <c r="G10" s="12" t="n"/>
+      <c r="H10" s="12" t="n"/>
+      <c r="I10" s="12" t="n"/>
+      <c r="J10" s="12" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="n"/>
-      <c r="B11" s="11" t="n"/>
-      <c r="C11" s="11" t="n"/>
-      <c r="D11" s="11" t="n"/>
-      <c r="E11" s="11" t="n"/>
-      <c r="F11" s="11" t="n"/>
-      <c r="G11" s="11" t="n"/>
-      <c r="H11" s="11" t="n"/>
-      <c r="I11" s="11" t="n"/>
-      <c r="J11" s="11" t="n"/>
-      <c r="K11" s="11" t="n"/>
+      <c r="A11" s="12" t="n"/>
+      <c r="B11" s="12" t="n"/>
+      <c r="C11" s="12" t="n"/>
+      <c r="D11" s="12" t="n"/>
+      <c r="E11" s="12" t="n"/>
+      <c r="F11" s="12" t="n"/>
+      <c r="G11" s="12" t="n"/>
+      <c r="H11" s="12" t="n"/>
+      <c r="I11" s="12" t="n"/>
+      <c r="J11" s="12" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="11" t="n"/>
-      <c r="B12" s="11" t="n"/>
-      <c r="C12" s="11" t="n"/>
-      <c r="D12" s="11" t="n"/>
-      <c r="E12" s="11" t="n"/>
-      <c r="F12" s="11" t="n"/>
-      <c r="G12" s="11" t="n"/>
-      <c r="H12" s="11" t="n"/>
-      <c r="I12" s="11" t="n"/>
-      <c r="J12" s="11" t="n"/>
-      <c r="K12" s="11" t="n"/>
+      <c r="A12" s="12" t="n"/>
+      <c r="B12" s="12" t="n"/>
+      <c r="C12" s="12" t="n"/>
+      <c r="D12" s="12" t="n"/>
+      <c r="E12" s="12" t="n"/>
+      <c r="F12" s="12" t="n"/>
+      <c r="G12" s="12" t="n"/>
+      <c r="H12" s="12" t="n"/>
+      <c r="I12" s="12" t="n"/>
+      <c r="J12" s="12" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="11" t="n"/>
-      <c r="B13" s="11" t="n"/>
-      <c r="C13" s="11" t="n"/>
-      <c r="D13" s="11" t="n"/>
-      <c r="E13" s="11" t="n"/>
-      <c r="F13" s="11" t="n"/>
-      <c r="G13" s="11" t="n"/>
-      <c r="H13" s="11" t="n"/>
-      <c r="I13" s="11" t="n"/>
-      <c r="J13" s="11" t="n"/>
-      <c r="K13" s="11" t="n"/>
+      <c r="A13" s="12" t="n"/>
+      <c r="B13" s="12" t="n"/>
+      <c r="C13" s="12" t="n"/>
+      <c r="D13" s="12" t="n"/>
+      <c r="E13" s="12" t="n"/>
+      <c r="F13" s="12" t="n"/>
+      <c r="G13" s="12" t="n"/>
+      <c r="H13" s="12" t="n"/>
+      <c r="I13" s="12" t="n"/>
+      <c r="J13" s="12" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="11" t="n"/>
-      <c r="B14" s="11" t="n"/>
-      <c r="C14" s="11" t="n"/>
-      <c r="D14" s="11" t="n"/>
-      <c r="E14" s="11" t="n"/>
-      <c r="F14" s="11" t="n"/>
-      <c r="G14" s="11" t="n"/>
-      <c r="H14" s="11" t="n"/>
-      <c r="I14" s="11" t="n"/>
-      <c r="J14" s="11" t="n"/>
-      <c r="K14" s="11" t="n"/>
+      <c r="A14" s="12" t="n"/>
+      <c r="B14" s="12" t="n"/>
+      <c r="C14" s="12" t="n"/>
+      <c r="D14" s="12" t="n"/>
+      <c r="E14" s="12" t="n"/>
+      <c r="F14" s="12" t="n"/>
+      <c r="G14" s="12" t="n"/>
+      <c r="H14" s="12" t="n"/>
+      <c r="I14" s="12" t="n"/>
+      <c r="J14" s="12" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="11" t="n"/>
-      <c r="B15" s="11" t="n"/>
-      <c r="C15" s="11" t="n"/>
-      <c r="D15" s="11" t="n"/>
-      <c r="E15" s="11" t="n"/>
-      <c r="F15" s="11" t="n"/>
-      <c r="G15" s="11" t="n"/>
-      <c r="H15" s="11" t="n"/>
-      <c r="I15" s="11" t="n"/>
-      <c r="J15" s="11" t="n"/>
-      <c r="K15" s="11" t="n"/>
+      <c r="A15" s="12" t="n"/>
+      <c r="B15" s="12" t="n"/>
+      <c r="C15" s="12" t="n"/>
+      <c r="D15" s="12" t="n"/>
+      <c r="E15" s="12" t="n"/>
+      <c r="F15" s="12" t="n"/>
+      <c r="G15" s="12" t="n"/>
+      <c r="H15" s="12" t="n"/>
+      <c r="I15" s="12" t="n"/>
+      <c r="J15" s="12" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="11" t="n"/>
-      <c r="B16" s="11" t="n"/>
-      <c r="C16" s="11" t="n"/>
-      <c r="D16" s="11" t="n"/>
-      <c r="E16" s="11" t="n"/>
-      <c r="F16" s="11" t="n"/>
-      <c r="G16" s="11" t="n"/>
-      <c r="H16" s="11" t="n"/>
-      <c r="I16" s="11" t="n"/>
-      <c r="J16" s="11" t="n"/>
-      <c r="K16" s="11" t="n"/>
+      <c r="A16" s="12" t="n"/>
+      <c r="B16" s="12" t="n"/>
+      <c r="C16" s="12" t="n"/>
+      <c r="D16" s="12" t="n"/>
+      <c r="E16" s="12" t="n"/>
+      <c r="F16" s="12" t="n"/>
+      <c r="G16" s="12" t="n"/>
+      <c r="H16" s="12" t="n"/>
+      <c r="I16" s="12" t="n"/>
+      <c r="J16" s="12" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="11" t="n"/>
-      <c r="B17" s="11" t="n"/>
-      <c r="C17" s="11" t="n"/>
-      <c r="D17" s="11" t="n"/>
-      <c r="E17" s="11" t="n"/>
-      <c r="F17" s="11" t="n"/>
-      <c r="G17" s="11" t="n"/>
-      <c r="H17" s="11" t="n"/>
-      <c r="I17" s="11" t="n"/>
-      <c r="J17" s="11" t="n"/>
-      <c r="K17" s="11" t="n"/>
+      <c r="A17" s="12" t="n"/>
+      <c r="B17" s="12" t="n"/>
+      <c r="C17" s="12" t="n"/>
+      <c r="D17" s="12" t="n"/>
+      <c r="E17" s="12" t="n"/>
+      <c r="F17" s="12" t="n"/>
+      <c r="G17" s="12" t="n"/>
+      <c r="H17" s="12" t="n"/>
+      <c r="I17" s="12" t="n"/>
+      <c r="J17" s="12" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="11" t="n"/>
-      <c r="B18" s="11" t="n"/>
-      <c r="C18" s="11" t="n"/>
-      <c r="D18" s="11" t="n"/>
-      <c r="E18" s="11" t="n"/>
-      <c r="F18" s="11" t="n"/>
-      <c r="G18" s="11" t="n"/>
-      <c r="H18" s="11" t="n"/>
-      <c r="I18" s="11" t="n"/>
-      <c r="J18" s="11" t="n"/>
-      <c r="K18" s="11" t="n"/>
+      <c r="A18" s="12" t="n"/>
+      <c r="B18" s="12" t="n"/>
+      <c r="C18" s="12" t="n"/>
+      <c r="D18" s="12" t="n"/>
+      <c r="E18" s="12" t="n"/>
+      <c r="F18" s="12" t="n"/>
+      <c r="G18" s="12" t="n"/>
+      <c r="H18" s="12" t="n"/>
+      <c r="I18" s="12" t="n"/>
+      <c r="J18" s="12" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="11" t="n"/>
-      <c r="B19" s="11" t="n"/>
-      <c r="C19" s="11" t="n"/>
-      <c r="D19" s="11" t="n"/>
-      <c r="E19" s="11" t="n"/>
-      <c r="F19" s="11" t="n"/>
-      <c r="G19" s="11" t="n"/>
-      <c r="H19" s="11" t="n"/>
-      <c r="I19" s="11" t="n"/>
-      <c r="J19" s="11" t="n"/>
-      <c r="K19" s="11" t="n"/>
+      <c r="A19" s="12" t="n"/>
+      <c r="B19" s="12" t="n"/>
+      <c r="C19" s="12" t="n"/>
+      <c r="D19" s="12" t="n"/>
+      <c r="E19" s="12" t="n"/>
+      <c r="F19" s="12" t="n"/>
+      <c r="G19" s="12" t="n"/>
+      <c r="H19" s="12" t="n"/>
+      <c r="I19" s="12" t="n"/>
+      <c r="J19" s="12" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="11" t="n"/>
-      <c r="B20" s="11" t="n"/>
-      <c r="C20" s="11" t="n"/>
-      <c r="D20" s="11" t="n"/>
-      <c r="E20" s="11" t="n"/>
-      <c r="F20" s="11" t="n"/>
-      <c r="G20" s="11" t="n"/>
-      <c r="H20" s="11" t="n"/>
-      <c r="I20" s="11" t="n"/>
-      <c r="J20" s="11" t="n"/>
-      <c r="K20" s="11" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="11" t="n"/>
-      <c r="B21" s="11" t="n"/>
-      <c r="C21" s="11" t="n"/>
-      <c r="D21" s="11" t="n"/>
-      <c r="E21" s="11" t="n"/>
-      <c r="F21" s="11" t="n"/>
-      <c r="G21" s="11" t="n"/>
-      <c r="H21" s="11" t="n"/>
-      <c r="I21" s="11" t="n"/>
-      <c r="J21" s="11" t="n"/>
-      <c r="K21" s="11" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="11" t="n"/>
-      <c r="B22" s="11" t="n"/>
-      <c r="C22" s="11" t="n"/>
-      <c r="D22" s="11" t="n"/>
-      <c r="E22" s="11" t="n"/>
-      <c r="F22" s="11" t="n"/>
-      <c r="G22" s="11" t="n"/>
-      <c r="H22" s="11" t="n"/>
-      <c r="I22" s="11" t="n"/>
-      <c r="J22" s="11" t="n"/>
-      <c r="K22" s="11" t="n"/>
+      <c r="A20" s="12" t="n"/>
+      <c r="B20" s="12" t="n"/>
+      <c r="C20" s="12" t="n"/>
+      <c r="D20" s="12" t="n"/>
+      <c r="E20" s="12" t="n"/>
+      <c r="F20" s="12" t="n"/>
+      <c r="G20" s="12" t="n"/>
+      <c r="H20" s="12" t="n"/>
+      <c r="I20" s="12" t="n"/>
+      <c r="J20" s="12" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="11" t="n"/>
-      <c r="B23" s="11" t="n"/>
-      <c r="C23" s="11" t="n"/>
-      <c r="D23" s="11" t="n"/>
-      <c r="E23" s="11" t="n"/>
-      <c r="F23" s="11" t="n"/>
-      <c r="G23" s="11" t="n"/>
-      <c r="H23" s="11" t="n"/>
-      <c r="I23" s="11" t="n"/>
-      <c r="J23" s="11" t="n"/>
-      <c r="K23" s="11" t="n"/>
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>* информация указывается только для дерматологических СИЗ</t>
+        </is>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" s="11" t="n"/>
-      <c r="B24" s="11" t="n"/>
-      <c r="C24" s="11" t="n"/>
-      <c r="D24" s="11" t="n"/>
-      <c r="E24" s="11" t="n"/>
-      <c r="F24" s="11" t="n"/>
-      <c r="G24" s="11" t="n"/>
-      <c r="H24" s="11" t="n"/>
-      <c r="I24" s="11" t="n"/>
-      <c r="J24" s="11" t="n"/>
-      <c r="K24" s="11" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="11" t="n"/>
-      <c r="B25" s="11" t="n"/>
-      <c r="C25" s="11" t="n"/>
-      <c r="D25" s="11" t="n"/>
-      <c r="E25" s="11" t="n"/>
-      <c r="F25" s="11" t="n"/>
-      <c r="G25" s="11" t="n"/>
-      <c r="H25" s="11" t="n"/>
-      <c r="I25" s="11" t="n"/>
-      <c r="J25" s="11" t="n"/>
-      <c r="K25" s="11" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>* информация указывается только для дерматологических СИЗ</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="A24" t="inlineStr">
         <is>
           <t>** информация указывается для всех СИЗ, кроме дерматологических СИЗ и СИЗ однократного применения</t>
         </is>
@@ -1229,11 +1142,11 @@
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="H3:K3"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="C3:F3"/>
+    <mergeCell ref="G3:J3"/>
+    <mergeCell ref="B3:B4"/>
     <mergeCell ref="A3:A4"/>
-    <mergeCell ref="B3:B4"/>
-    <mergeCell ref="H1:K1"/>
-    <mergeCell ref="C3:G3"/>
   </mergeCells>
   <pageMargins left="0.4" right="0.4" top="0.6" bottom="0.4" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>

</xml_diff>